<commit_message>
AU capacity: a run's snapshot replaces the same month's saved row (no stale columns); saved Oct/26 row repaired
</commit_message>
<xml_diff>
--- a/output/Data and Chart Outputs/au_power_capacity.xlsx
+++ b/output/Data and Chart Outputs/au_power_capacity.xlsx
@@ -791,7 +791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A13"/>
+  <dimension ref="A1:A11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -839,38 +839,36 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>COVERAGE</t>
+        </is>
+      </c>
+    </row>
     <row r="8">
-      <c r="A8" s="1" t="inlineStr">
-        <is>
-          <t>COVERAGE</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>NEM (QLD, NSW, VIC, SA, TAS) + WA's WEM. Rooftop solar, NT and off-grid plant not included. Series starts with the first run (Oct 2026) - AEMO publishes no capacity history in these lists.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>NEM (QLD, NSW, VIC, SA, TAS) + WA's WEM. Rooftop solar, NT and off-grid plant not included. Series starts with the first run (Oct 2026) - AEMO publishes no capacity history in these lists.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>SOURCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>AEMO NEM Registration and Exemption List: https://www.aemo.com.au/-/media/Files/Electricity/NEM/Participant_Information/NEM-Registration-and-Exemption-List.xls; AEMO WA facilities list: https://data.wa.aemo.com.au/public/public-data/datafiles/facilities/facilities.csv</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>SOURCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>AEMO NEM Registration and Exemption List: https://www.aemo.com.au/-/media/Files/Electricity/NEM/Participant_Information/NEM-Registration-and-Exemption-List.xls; AEMO WA facilities list: https://data.wa.aemo.com.au/public/public-data/datafiles/facilities/facilities.csv</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>https://aemo.com.au/en/energy-systems/electricity/national-electricity-market-nem/participate-in-the-market/registration</t>
         </is>
@@ -921,17 +919,17 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Nuclear &amp; other</t>
+          <t>Battery storage</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Battery storage</t>
+          <t>Hydro</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Hydro</t>
+          <t>Pumped storage</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -957,16 +955,16 @@
         <v>15.072</v>
       </c>
       <c r="F2" t="n">
-        <v>14.8416</v>
+        <v>13.7294</v>
       </c>
       <c r="G2" t="n">
-        <v>13.7294</v>
+        <v>7.3899</v>
       </c>
       <c r="H2" t="n">
-        <v>7.3899</v>
+        <v>0.7059</v>
       </c>
       <c r="I2" t="n">
-        <v>1.2735</v>
+        <v>0.5676</v>
       </c>
     </row>
   </sheetData>
@@ -981,7 +979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1040,11 +1038,6 @@
           <t>Pumped_storage_MW</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
-        <is>
-          <t>Other_MW</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="n">
@@ -1079,9 +1072,6 @@
       </c>
       <c r="K2" t="n">
         <v>705.9</v>
-      </c>
-      <c r="L2" t="n">
-        <v>14841.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>